<commit_message>
Case Study Input update
</commit_message>
<xml_diff>
--- a/Case_Study/Sample_use_case_setup.xlsx
+++ b/Case_Study/Sample_use_case_setup.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jbrauch\Desktop\HYPSTAT open sourcing\HYPSTAT\Case_Study\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yli6/Desktop/NREL/Project/HYPSTAT/HYPSTAT_github/HYPSTAT/Case_Study/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6572167F-6DB3-4143-ADA7-C1D4743DA91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{319E2148-11A5-854C-888C-1292BB0B942B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8240C5C8-55BB-784E-92A0-705DB0403669}"/>
+    <workbookView xWindow="11980" yWindow="4400" windowWidth="23260" windowHeight="12580" xr2:uid="{8240C5C8-55BB-784E-92A0-705DB0403669}"/>
   </bookViews>
   <sheets>
     <sheet name="Zone" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="79">
   <si>
     <t>Node</t>
   </si>
@@ -256,6 +256,27 @@
   </si>
   <si>
     <t>YES (Wholesale, higher)</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>North Carolina</t>
+  </si>
+  <si>
+    <t>Colorado</t>
+  </si>
+  <si>
+    <t>Washington</t>
+  </si>
+  <si>
+    <t>Sample State</t>
+  </si>
+  <si>
+    <t>Texas</t>
+  </si>
+  <si>
+    <t>Florida</t>
   </si>
 </sst>
 </file>
@@ -2044,15 +2065,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{773A3E98-2DE2-3246-BBBC-A7EFDC583254}">
-  <dimension ref="A1:L21"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="17.69921875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="29.19921875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.59765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2089,8 +2110,11 @@
       <c r="L1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2127,8 +2151,11 @@
       <c r="L2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2165,8 +2192,11 @@
       <c r="L3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2203,8 +2233,11 @@
       <c r="L4" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -2241,8 +2274,11 @@
       <c r="L5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -2279,8 +2315,11 @@
       <c r="L6" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -2317,33 +2356,36 @@
       <c r="L7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="H16" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H17" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H18" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H19" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H20" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="8:8" x14ac:dyDescent="0.2">
       <c r="H21" t="s">
         <v>18</v>
       </c>
@@ -2357,15 +2399,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9634E36E-1C52-4E1E-8DF9-F0779669CEEC}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.59765625" customWidth="1"/>
-    <col min="2" max="2" width="14.69921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="56.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.8984375" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="56.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2379,7 +2421,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2393,7 +2435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2407,7 +2449,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2421,7 +2463,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -2435,7 +2477,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -2449,7 +2491,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -2471,13 +2513,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4290B951-8F0C-5349-9F5D-132B582F7790}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.69921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -2485,7 +2527,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>14</v>
       </c>
@@ -2493,7 +2535,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>14</v>
       </c>
@@ -2501,7 +2543,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>14</v>
       </c>
@@ -2509,7 +2551,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>14</v>
       </c>
@@ -2517,7 +2559,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>14</v>
       </c>
@@ -2525,7 +2567,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>16</v>
       </c>
@@ -2533,7 +2575,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>17</v>
       </c>
@@ -2541,7 +2583,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>17</v>
       </c>
@@ -2549,7 +2591,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>35</v>
       </c>
@@ -2557,7 +2599,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>35</v>
       </c>
@@ -2573,13 +2615,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2155F4B6-E3DC-3443-8726-D23849DFF292}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="14.69921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="49.296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="49.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>13</v>
       </c>
@@ -2590,7 +2632,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>14</v>
       </c>
@@ -2601,7 +2643,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>14</v>
       </c>
@@ -2612,7 +2654,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>14</v>
       </c>
@@ -2623,7 +2665,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>14</v>
       </c>
@@ -2634,7 +2676,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>14</v>
       </c>
@@ -2645,7 +2687,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>16</v>
       </c>
@@ -2656,7 +2698,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>17</v>
       </c>
@@ -2667,7 +2709,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>17</v>
       </c>
@@ -2678,7 +2720,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>35</v>
       </c>
@@ -2689,7 +2731,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>35</v>
       </c>
@@ -2708,14 +2750,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E88A2DE3-4377-5F45-9DB5-C20D6C029B92}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.3984375" customWidth="1"/>
-    <col min="3" max="3" width="19.296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -2729,7 +2771,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -2743,7 +2785,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -2757,7 +2799,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2771,7 +2813,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -2779,7 +2821,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -2793,7 +2835,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -2807,7 +2849,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>46</v>
       </c>
@@ -2821,7 +2863,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -2835,7 +2877,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
study background writeup and input folders
</commit_message>
<xml_diff>
--- a/Case_Study/Sample_use_case_setup.xlsx
+++ b/Case_Study/Sample_use_case_setup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yli6/Desktop/NREL/Project/HYPSTAT/HYPSTAT_github/HYPSTAT/Case_Study/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{319E2148-11A5-854C-888C-1292BB0B942B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06EC4394-DF90-C74D-A29A-34D68012F741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11980" yWindow="4400" windowWidth="23260" windowHeight="12580" xr2:uid="{8240C5C8-55BB-784E-92A0-705DB0403669}"/>
   </bookViews>
@@ -299,7 +299,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -335,6 +335,12 @@
         <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -364,7 +370,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -372,6 +378,8 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -2065,12 +2073,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{773A3E98-2DE2-3246-BBBC-A7EFDC583254}">
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.6640625" customWidth="1"/>
     <col min="8" max="8" width="29.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
@@ -2360,35 +2369,175 @@
         <v>78</v>
       </c>
     </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="7"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="7"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="7"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="7"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="7"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="7"/>
+    </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="7"/>
       <c r="H16" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="7"/>
       <c r="H17" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="7"/>
       <c r="H18" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="8:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="7"/>
       <c r="H19" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="8:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="7"/>
       <c r="H20" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="7"/>
       <c r="H21" t="s">
         <v>18</v>
       </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="7"/>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="7"/>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>